<commit_message>
Changed power supply. Included THT in SMD assembly. Regenerated Project Outputs
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_A_MAX11331_Adapter/BOM/BOM_UltraZohm_Analog_Adapter_MAX11331_2v01.xlsx
+++ b/Project Outputs for UZ_A_MAX11331_Adapter/BOM/BOM_UltraZohm_Analog_Adapter_MAX11331_2v01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UltraZohm\UZ_A_MAX11331_Adapter\Project Outputs for UZ_A_MAX11331_Adapter\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\Altium\UltraZOhm\UZ_A_MAX1131_Adapter\Project Outputs for UZ_A_MAX11331_Adapter\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1EEEC44-D079-4469-923C-DCE295D20ED4}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2E9F32F-DABD-46CE-9676-D3B9AC65031C}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2460" windowWidth="14670" windowHeight="8325" xr2:uid="{68AD2743-5D5E-4BB5-BC1E-028ABE70507C}"/>
+    <workbookView xWindow="1500" yWindow="180" windowWidth="21600" windowHeight="11385" xr2:uid="{C02DD4BB-3304-4F75-86B1-FE279DA5D586}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UltraZohm_Analog_Adapter_MA" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="155">
   <si>
     <t>Name</t>
   </si>
@@ -117,7 +117,7 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>C1, C2, C3A, C3B, C3C, C4A, C4B, C4C, C10, C13, C18, C19, C20, C21, C22, C23, C24, C25</t>
+    <t>C1, C2, C3A, C3B, C3C, C4A, C4B, C4C, C6, C10, C13, C18, C19, C20, C21, C22, C23, C24, C25</t>
   </si>
   <si>
     <t>Capacitor</t>
@@ -147,66 +147,54 @@
     <t>C0603C104M5RACTU</t>
   </si>
   <si>
-    <t>2.2nF</t>
-  </si>
-  <si>
-    <t>C6</t>
+    <t>68µF</t>
+  </si>
+  <si>
+    <t>C8, C9</t>
+  </si>
+  <si>
+    <t>WCAP-ATG8 THT Aluminum Electrolytic Capacitors, D6.3mm x L11mm, 68uF, +/-20%, 35VDC</t>
+  </si>
+  <si>
+    <t>+/-20%</t>
+  </si>
+  <si>
+    <t>WCAP-ATG8_6.3x11</t>
+  </si>
+  <si>
+    <t>732-8736-1-ND</t>
+  </si>
+  <si>
+    <t>860010573006</t>
+  </si>
+  <si>
+    <t>10µF</t>
+  </si>
+  <si>
+    <t>C11, C12</t>
+  </si>
+  <si>
+    <t>35 V</t>
+  </si>
+  <si>
+    <t>490-9964-1-ND</t>
+  </si>
+  <si>
+    <t>Murata</t>
+  </si>
+  <si>
+    <t>GRM319R6YA106KA12D</t>
+  </si>
+  <si>
+    <t>1µF</t>
+  </si>
+  <si>
+    <t>C14, C15, C16, C17</t>
   </si>
   <si>
     <t>Capacitor Ceramic</t>
   </si>
   <si>
-    <t>50V</t>
-  </si>
-  <si>
-    <t>399-17586-6-ND</t>
-  </si>
-  <si>
-    <t>C0603C222K5RAC7411</t>
-  </si>
-  <si>
-    <t>1.2nF</t>
-  </si>
-  <si>
-    <t>C7</t>
-  </si>
-  <si>
-    <t>5%</t>
-  </si>
-  <si>
-    <t>CG0</t>
-  </si>
-  <si>
-    <t>399-7851-6-ND</t>
-  </si>
-  <si>
-    <t>C0603C122K5RACTU</t>
-  </si>
-  <si>
-    <t>10µF</t>
-  </si>
-  <si>
-    <t>C11, C12</t>
-  </si>
-  <si>
-    <t>35 V</t>
-  </si>
-  <si>
-    <t>490-9964-1-ND</t>
-  </si>
-  <si>
-    <t>Murata</t>
-  </si>
-  <si>
-    <t>GRM319R6YA106KA12D</t>
-  </si>
-  <si>
-    <t>1µF</t>
-  </si>
-  <si>
-    <t>C14, C16, C17</t>
-  </si>
-  <si>
     <t>50 V</t>
   </si>
   <si>
@@ -216,18 +204,6 @@
     <t>C0603C105K3RACTU</t>
   </si>
   <si>
-    <t>91pF</t>
-  </si>
-  <si>
-    <t>C15</t>
-  </si>
-  <si>
-    <t>490-1426-1-ND</t>
-  </si>
-  <si>
-    <t>GRM1885C1H910JA01D</t>
-  </si>
-  <si>
     <t>Bright Green, 2V</t>
   </si>
   <si>
@@ -240,7 +216,7 @@
     <t>WL-SMCW_0603_H=0.7mm</t>
   </si>
   <si>
-    <t>732-4980-6-ND</t>
+    <t>732-4980-1-ND</t>
   </si>
   <si>
     <t>150060VS75000</t>
@@ -276,25 +252,22 @@
     <t>150060SS75000</t>
   </si>
   <si>
-    <t>33µH</t>
+    <t>15mH</t>
   </si>
   <si>
     <t>L1</t>
   </si>
   <si>
-    <t>SMT power Inductor, 33µH, 225m DRC</t>
-  </si>
-  <si>
-    <t>Inductor 5030</t>
-  </si>
-  <si>
-    <t>587-3458-6-ND</t>
-  </si>
-  <si>
-    <t>Taiyo Yuden</t>
-  </si>
-  <si>
-    <t>NRS5030T330MMGJ</t>
+    <t>SMT power Inductor, 15uH, 40m DRC</t>
+  </si>
+  <si>
+    <t>SMT_inductor_1050_Performance</t>
+  </si>
+  <si>
+    <t>811-3837-1-ND</t>
+  </si>
+  <si>
+    <t>48150SC</t>
   </si>
   <si>
     <t>0</t>
@@ -324,7 +297,7 @@
     <t>10k</t>
   </si>
   <si>
-    <t>R4, R5, R6, R7, R10, R11, R12, R13, R15, R16, R17, R18, R19, R20, R28, R31, R32, R33, R34, R35, R36</t>
+    <t>R4, R5, R6, R7, R10, R11, R12, R13, R15, R16, R17, R18, R19, R20, R31, R32, R33, R34, R35, R36</t>
   </si>
   <si>
     <t>311-10.0KHRCT-ND</t>
@@ -342,6 +315,9 @@
     <t>311-100HRCT-ND</t>
   </si>
   <si>
+    <t>Mepco Philips</t>
+  </si>
+  <si>
     <t>RC0603FR-07100RL</t>
   </si>
   <si>
@@ -357,43 +333,28 @@
     <t>RC0603FR-072M2L</t>
   </si>
   <si>
-    <t>200k</t>
+    <t>100k</t>
   </si>
   <si>
     <t>R26</t>
   </si>
   <si>
-    <t>311-200KHRDKR-ND</t>
-  </si>
-  <si>
-    <t>RC0603FR-07200KL</t>
-  </si>
-  <si>
-    <t>115k</t>
+    <t>311-100KHRDKR-ND</t>
+  </si>
+  <si>
+    <t>RC0603FR-07100KL</t>
+  </si>
+  <si>
+    <t>38.3k</t>
   </si>
   <si>
     <t>R27</t>
   </si>
   <si>
-    <t>311-115KHRDKR-ND</t>
-  </si>
-  <si>
-    <t>RC0603FR-07115KL</t>
-  </si>
-  <si>
-    <t>100k</t>
-  </si>
-  <si>
-    <t>R29</t>
-  </si>
-  <si>
-    <t>311-100KHRCT-ND</t>
-  </si>
-  <si>
-    <t>Mepco Philips</t>
-  </si>
-  <si>
-    <t>RC0603FR-07100KL</t>
+    <t>311-38.3KHRCT-ND</t>
+  </si>
+  <si>
+    <t>RC0603FR-0738K3L</t>
   </si>
   <si>
     <t>220</t>
@@ -474,25 +435,22 @@
     <t>ADN4666ARUZ</t>
   </si>
   <si>
-    <t>buck converter</t>
+    <t>Buck Converter</t>
   </si>
   <si>
     <t>U5</t>
   </si>
   <si>
-    <t>100V Input, 0.5A Synchronous Buck DC/DC Converter with Ultra-low Iq</t>
+    <t>3.8V to 36V, 2A synchronous step-down converter</t>
   </si>
   <si>
     <t>SOIC127P600X170_HS-9N</t>
   </si>
   <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>296-LM5163HQDDARQ1CT-ND</t>
-  </si>
-  <si>
-    <t>LM5163HQDDARQ1</t>
+    <t>296-48841-ND</t>
+  </si>
+  <si>
+    <t>LMR33620ADDA</t>
   </si>
   <si>
     <t>1.8V LDO</t>
@@ -514,6 +472,36 @@
   </si>
   <si>
     <t>TLV1117-15IDCYR</t>
+  </si>
+  <si>
+    <t>2x8 Pin</t>
+  </si>
+  <si>
+    <t>X2A, X2B, X2C</t>
+  </si>
+  <si>
+    <t>Dual Row, 2x8 Shrouded IDC Header with Ejectors 50 mil pitch</t>
+  </si>
+  <si>
+    <t>EHF-108-01-F-D</t>
+  </si>
+  <si>
+    <t>SAM9265-ND</t>
+  </si>
+  <si>
+    <t>Samtec</t>
+  </si>
+  <si>
+    <t>IPL1-102-01-L-D-K</t>
+  </si>
+  <si>
+    <t>X3, X4, X5</t>
+  </si>
+  <si>
+    <t>2.54mm Double Row Terminal Assembly, Right-Angled</t>
+  </si>
+  <si>
+    <t>SAM10565-ND</t>
   </si>
 </sst>
 </file>
@@ -584,7 +572,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -600,7 +588,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -895,24 +883,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1A2C623-9DFE-44CF-AC9A-FDBFE51441F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7304ADFE-990B-457E-A256-DD854A4BAA48}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="8" width="16.5703125" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1"/>
-    <col min="12" max="14" width="16.5703125" customWidth="1"/>
-    <col min="15" max="15" width="10.5703125" customWidth="1"/>
-    <col min="16" max="16" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
+    <col min="5" max="8" width="16.7109375" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" customWidth="1"/>
+    <col min="12" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -965,7 +953,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
@@ -1051,13 +1039,13 @@
         <v>3.5000000000000003E-2</v>
       </c>
       <c r="O3" s="4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P3" s="4">
-        <v>0.63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.66500000000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>36</v>
       </c>
@@ -1070,70 +1058,66 @@
       <c r="D4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>28</v>
-      </c>
+      <c r="E4" s="4"/>
       <c r="F4" s="3" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>31</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="H4" s="4"/>
       <c r="I4" s="3" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N4" s="4">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="O4" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P4" s="4">
-        <v>0.1</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>42</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>21</v>
@@ -1142,181 +1126,165 @@
         <v>46</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N5" s="4">
-        <v>0.1</v>
+        <v>0.34</v>
       </c>
       <c r="O5" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P5" s="4">
-        <v>0.1</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>48</v>
-      </c>
       <c r="D6" s="3" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>29</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>31</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N6" s="4">
-        <v>0.34</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="O6" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4">
-        <v>0.68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>1.1200000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>54</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C7" s="4"/>
       <c r="D7" s="3" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
       <c r="I7" s="3" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="N7" s="4">
-        <v>0.28000000000000003</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O7" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P7" s="4">
-        <v>0.84</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>59</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C8" s="4"/>
       <c r="D8" s="3" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>45</v>
-      </c>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
       <c r="I8" s="3" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="N8" s="4">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="O8" s="4">
         <v>1</v>
       </c>
       <c r="P8" s="4">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>28</v>
@@ -1325,19 +1293,19 @@
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="3" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="N9" s="4">
         <v>0.14000000000000001</v>
@@ -1349,155 +1317,163 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C10" s="4"/>
+        <v>72</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="D10" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>28</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="3" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="N10" s="4">
-        <v>0.16</v>
+        <v>1.36</v>
       </c>
       <c r="O10" s="4">
         <v>1</v>
       </c>
       <c r="P10" s="4">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C11" s="4"/>
+        <v>78</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="D11" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="4"/>
+      <c r="F11" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="3" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="N11" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="O11" s="4">
         <v>1</v>
       </c>
       <c r="P11" s="4">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="E12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K12" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="L12" s="3" t="s">
-        <v>84</v>
-      </c>
       <c r="M12" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="N12" s="4">
-        <v>0.33</v>
+        <v>2.4E-2</v>
       </c>
       <c r="O12" s="4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="P12" s="4">
-        <v>0.33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="3" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>21</v>
@@ -1512,16 +1488,16 @@
         <v>93</v>
       </c>
       <c r="N13" s="4">
-        <v>0.1</v>
+        <v>2.4E-2</v>
       </c>
       <c r="O13" s="4">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="P13" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>0.38400000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>94</v>
       </c>
@@ -1532,18 +1508,18 @@
         <v>94</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="3" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>21</v>
@@ -1552,22 +1528,22 @@
         <v>96</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>97</v>
       </c>
       <c r="N14" s="4">
-        <v>2.4E-2</v>
+        <v>0.1</v>
       </c>
       <c r="O14" s="4">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="P14" s="4">
-        <v>0.504</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>98</v>
       </c>
@@ -1578,18 +1554,18 @@
         <v>98</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="3" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>21</v>
@@ -1598,19 +1574,19 @@
         <v>100</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>101</v>
       </c>
       <c r="N15" s="4">
-        <v>2.4E-2</v>
+        <v>0.1</v>
       </c>
       <c r="O15" s="4">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="P15" s="4">
-        <v>0.38400000000000001</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
@@ -1624,18 +1600,18 @@
         <v>102</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="3" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>21</v>
@@ -1644,7 +1620,7 @@
         <v>104</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>105</v>
@@ -1670,18 +1646,18 @@
         <v>106</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="3" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>21</v>
@@ -1690,7 +1666,7 @@
         <v>108</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>109</v>
@@ -1716,18 +1692,18 @@
         <v>110</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="3" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>21</v>
@@ -1736,7 +1712,7 @@
         <v>112</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>113</v>
@@ -1751,343 +1727,291 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="210" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>114</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>114</v>
-      </c>
+      <c r="C19" s="4"/>
       <c r="D19" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>89</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="3" t="s">
-        <v>90</v>
+        <v>117</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="N19" s="4">
-        <v>0.1</v>
+        <v>1.39</v>
       </c>
       <c r="O19" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P19" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>6.95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>119</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="C20" s="4"/>
       <c r="D20" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>89</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="3" t="s">
-        <v>90</v>
+        <v>117</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="N20" s="4">
-        <v>0.1</v>
+        <v>3.34</v>
       </c>
       <c r="O20" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P20" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>10.02</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>123</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="C21" s="4"/>
       <c r="D21" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>89</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="3" t="s">
-        <v>90</v>
+        <v>117</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K21" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="L21" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="L21" s="3" t="s">
-        <v>92</v>
-      </c>
       <c r="M21" s="3" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="N21" s="4">
-        <v>0.1</v>
+        <v>3.34</v>
       </c>
       <c r="O21" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P21" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" ht="225" x14ac:dyDescent="0.25">
+        <v>10.02</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="3" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="N22" s="4">
-        <v>1.39</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="O22" s="4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P22" s="4">
-        <v>6.95</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="3" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>21</v>
+        <v>142</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="N23" s="4">
-        <v>3.34</v>
+        <v>0.71</v>
       </c>
       <c r="O23" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P23" s="4">
-        <v>10.02</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="3" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="N24" s="4">
-        <v>3.34</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="O24" s="4">
         <v>3</v>
       </c>
       <c r="P24" s="4">
-        <v>10.02</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="105" x14ac:dyDescent="0.25">
+        <v>14.55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C25" s="4"/>
+        <v>152</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>151</v>
+      </c>
       <c r="D25" s="3" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>149</v>
+        <v>21</v>
       </c>
       <c r="K25" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>150</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>132</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="N25" s="4"/>
+      <c r="N25" s="4">
+        <v>3.64</v>
+      </c>
       <c r="O25" s="4">
-        <v>1</v>
-      </c>
-      <c r="P25" s="4"/>
-    </row>
-    <row r="26" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="L26" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="M26" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="N26" s="4">
-        <v>0.71</v>
-      </c>
-      <c r="O26" s="4">
-        <v>1</v>
-      </c>
-      <c r="P26" s="4">
-        <v>0.71</v>
+        <v>3</v>
+      </c>
+      <c r="P25" s="4">
+        <v>10.92</v>
       </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="35" orientation="landscape" horizontalDpi="4294967292" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="32" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated value 15uH instead 15mH in power supply. Update resistors in formula for power supply Added clock return components in SMD_assembly Regenerate fabrication outputs
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_A_MAX11331_Adapter/BOM/BOM_UltraZohm_Analog_Adapter_MAX11331_2v01.xlsx
+++ b/Project Outputs for UZ_A_MAX11331_Adapter/BOM/BOM_UltraZohm_Analog_Adapter_MAX11331_2v01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\Altium\UltraZOhm\UZ_A_MAX1131_Adapter\Project Outputs for UZ_A_MAX11331_Adapter\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Altium_projects\UltraZohm\UZ_A_MAX11331_Adapter\Project Outputs for UZ_A_MAX11331_Adapter\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2E9F32F-DABD-46CE-9676-D3B9AC65031C}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{88B6FD52-1CCA-4217-9F99-9EF3B84AFED2}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="180" windowWidth="21600" windowHeight="11385" xr2:uid="{C02DD4BB-3304-4F75-86B1-FE279DA5D586}"/>
+    <workbookView xWindow="1020" yWindow="1290" windowWidth="21600" windowHeight="11505" xr2:uid="{EBBBBB7E-777F-415E-838D-6B2A33DD75B6}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UltraZohm_Analog_Adapter_MA" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="161">
   <si>
     <t>Name</t>
   </si>
@@ -252,7 +252,7 @@
     <t>150060SS75000</t>
   </si>
   <si>
-    <t>15mH</t>
+    <t>15uH</t>
   </si>
   <si>
     <t>L1</t>
@@ -264,12 +264,12 @@
     <t>SMT_inductor_1050_Performance</t>
   </si>
   <si>
+    <t>Digikey</t>
+  </si>
+  <si>
     <t>811-3837-1-ND</t>
   </si>
   <si>
-    <t>48150SC</t>
-  </si>
-  <si>
     <t>0</t>
   </si>
   <si>
@@ -433,6 +433,24 @@
   </si>
   <si>
     <t>ADN4666ARUZ</t>
+  </si>
+  <si>
+    <t>Signle LVDS receiver</t>
+  </si>
+  <si>
+    <t>U4A, U4B, U4C</t>
+  </si>
+  <si>
+    <t>Single, 3V, CMOS, LVDS High Speed Differential Receiver</t>
+  </si>
+  <si>
+    <t>SOIC127P600X170_HS-9N_no_THP</t>
+  </si>
+  <si>
+    <t>ADN4662BRZ-ND</t>
+  </si>
+  <si>
+    <t>ADN4662BRZ</t>
   </si>
   <si>
     <t>Buck Converter</t>
@@ -572,7 +590,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -588,7 +606,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -883,24 +901,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7304ADFE-990B-457E-A256-DD854A4BAA48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{134B0142-2D34-4EF2-A9BF-F6847C71B7F5}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" customWidth="1"/>
-    <col min="5" max="8" width="16.7109375" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="12.42578125" customWidth="1"/>
-    <col min="11" max="11" width="15.85546875" customWidth="1"/>
-    <col min="12" max="14" width="16.7109375" customWidth="1"/>
-    <col min="15" max="15" width="10.7109375" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="8" width="16.5703125" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="12" max="14" width="16.5703125" customWidth="1"/>
+    <col min="15" max="15" width="10.5703125" customWidth="1"/>
+    <col min="16" max="16" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -953,7 +971,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
@@ -1338,26 +1356,18 @@
         <v>74</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="M10" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="N10" s="4">
-        <v>1.36</v>
-      </c>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
       <c r="O10" s="4">
         <v>1</v>
       </c>
-      <c r="P10" s="4">
-        <v>1.36</v>
-      </c>
+      <c r="P10" s="4"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
@@ -1727,7 +1737,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="210" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="225" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>114</v>
       </c>
@@ -1807,7 +1817,7 @@
         <v>10.02</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>127</v>
       </c>
@@ -1872,19 +1882,19 @@
         <v>136</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>137</v>
       </c>
       <c r="N22" s="4">
-        <v>2.4300000000000002</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="O22" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P22" s="4">
-        <v>2.4300000000000002</v>
+        <v>6.66</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="75" x14ac:dyDescent="0.25">
@@ -1906,77 +1916,75 @@
         <v>141</v>
       </c>
       <c r="J23" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K23" s="3" t="s">
         <v>142</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>143</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>119</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="N23" s="4">
-        <v>0.71</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="O23" s="4">
         <v>1</v>
       </c>
       <c r="P23" s="4">
-        <v>0.71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>145</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>146</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="J24" s="3" t="s">
         <v>148</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>21</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>149</v>
       </c>
       <c r="L24" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="M24" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="M24" s="3" t="s">
-        <v>148</v>
-      </c>
       <c r="N24" s="4">
-        <v>4.8499999999999996</v>
+        <v>0.71</v>
       </c>
       <c r="O24" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P24" s="4">
-        <v>14.55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>151</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>151</v>
-      </c>
+      <c r="C25" s="4"/>
       <c r="D25" s="3" t="s">
         <v>153</v>
       </c>
@@ -1985,33 +1993,75 @@
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K25" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="M25" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="L25" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="M25" s="3" t="s">
-        <v>151</v>
-      </c>
       <c r="N25" s="4">
-        <v>3.64</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="O25" s="4">
         <v>3</v>
       </c>
       <c r="P25" s="4">
+        <v>14.55</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="N26" s="4">
+        <v>3.64</v>
+      </c>
+      <c r="O26" s="4">
+        <v>3</v>
+      </c>
+      <c r="P26" s="4">
         <v>10.92</v>
       </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="32" orientation="landscape" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="30" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added orientation marking, added R8,9,14 C5 to SMD Assembly
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_A_MAX11331_Adapter/BOM/BOM_UltraZohm_Analog_Adapter_MAX11331_2v01.xlsx
+++ b/Project Outputs for UZ_A_MAX11331_Adapter/BOM/BOM_UltraZohm_Analog_Adapter_MAX11331_2v01.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Altium_projects\UltraZohm\UZ_A_MAX11331_Adapter\Project Outputs for UZ_A_MAX11331_Adapter\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hm-kreppel\Documents\Altium Projects\uz_a_max11331_adapter\Project Outputs for UZ_A_MAX11331_Adapter\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88B6FD52-1CCA-4217-9F99-9EF3B84AFED2}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1020" yWindow="1290" windowWidth="21600" windowHeight="11505" xr2:uid="{EBBBBB7E-777F-415E-838D-6B2A33DD75B6}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="11565"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UltraZohm_Analog_Adapter_MA" sheetId="1" r:id="rId1"/>
@@ -18,26 +17,17 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">BOM_UltraZohm_Analog_Adapter_MA!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="163">
   <si>
     <t>Name</t>
   </si>
@@ -117,7 +107,7 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>C1, C2, C3A, C3B, C3C, C4A, C4B, C4C, C6, C10, C13, C18, C19, C20, C21, C22, C23, C24, C25</t>
+    <t>C1, C2, C3A, C3B, C3C, C4A, C4B, C4C, C5A, C5B, C5C, C6, C10, C13, C18, C19, C20, C21, C22, C23, C24, C25</t>
   </si>
   <si>
     <t>Capacitor</t>
@@ -304,6 +294,12 @@
   </si>
   <si>
     <t>RC0603FR-0710KL</t>
+  </si>
+  <si>
+    <t>0R</t>
+  </si>
+  <si>
+    <t>R8, R9, R14</t>
   </si>
   <si>
     <t>100R</t>
@@ -525,7 +521,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -590,7 +586,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -606,7 +602,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -622,7 +618,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -634,7 +630,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -681,23 +677,6 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -733,23 +712,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -901,24 +863,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{134B0142-2D34-4EF2-A9BF-F6847C71B7F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="8" width="16.5703125" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1"/>
-    <col min="12" max="14" width="16.5703125" customWidth="1"/>
-    <col min="15" max="15" width="10.5703125" customWidth="1"/>
-    <col min="16" max="16" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
+    <col min="5" max="8" width="16.7109375" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" customWidth="1"/>
+    <col min="12" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -971,7 +933,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
@@ -1013,7 +975,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>25</v>
       </c>
@@ -1057,10 +1019,10 @@
         <v>3.5000000000000003E-2</v>
       </c>
       <c r="O3" s="4">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="P3" s="4">
-        <v>0.66500000000000004</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="135" x14ac:dyDescent="0.25">
@@ -1461,7 +1423,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>89</v>
       </c>
@@ -1489,33 +1451,33 @@
         <v>21</v>
       </c>
       <c r="K13" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="N13" s="4">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="O13" s="4">
+        <v>3</v>
+      </c>
+      <c r="P13" s="4">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="L13" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="M13" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="N13" s="4">
-        <v>2.4E-2</v>
-      </c>
-      <c r="O13" s="4">
-        <v>16</v>
-      </c>
-      <c r="P13" s="4">
-        <v>0.38400000000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="C14" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>79</v>
@@ -1535,33 +1497,33 @@
         <v>21</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="N14" s="4">
-        <v>0.1</v>
+        <v>2.4E-2</v>
       </c>
       <c r="O14" s="4">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="P14" s="4">
-        <v>0.1</v>
+        <v>0.38400000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>79</v>
@@ -1581,13 +1543,13 @@
         <v>21</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>83</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="N15" s="4">
         <v>0.1</v>
@@ -1601,13 +1563,13 @@
     </row>
     <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>79</v>
@@ -1627,13 +1589,13 @@
         <v>21</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>83</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="N16" s="4">
         <v>0.1</v>
@@ -1647,13 +1609,13 @@
     </row>
     <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>79</v>
@@ -1673,13 +1635,13 @@
         <v>21</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>83</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="N17" s="4">
         <v>0.1</v>
@@ -1693,13 +1655,13 @@
     </row>
     <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>79</v>
@@ -1719,13 +1681,13 @@
         <v>21</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>83</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="N18" s="4">
         <v>0.1</v>
@@ -1737,115 +1699,121 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="225" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C19" s="4"/>
+        <v>113</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>112</v>
+      </c>
       <c r="D19" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+        <v>79</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="M19" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="N19" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="O19" s="4">
+        <v>1</v>
+      </c>
+      <c r="P19" s="4">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="210" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="N19" s="4">
-        <v>1.39</v>
-      </c>
-      <c r="O19" s="4">
-        <v>5</v>
-      </c>
-      <c r="P19" s="4">
-        <v>6.95</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>122</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="3" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K20" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="N20" s="4">
+        <v>1.39</v>
+      </c>
+      <c r="O20" s="4">
+        <v>5</v>
+      </c>
+      <c r="P20" s="4">
+        <v>6.95</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="N20" s="4">
-        <v>3.34</v>
-      </c>
-      <c r="O20" s="4">
-        <v>3</v>
-      </c>
-      <c r="P20" s="4">
-        <v>10.02</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>128</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="N21" s="4">
         <v>3.34</v>
@@ -1857,205 +1825,245 @@
         <v>10.02</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="3" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="N22" s="4">
-        <v>2.2200000000000002</v>
+        <v>3.34</v>
       </c>
       <c r="O22" s="4">
         <v>3</v>
       </c>
       <c r="P22" s="4">
-        <v>6.66</v>
+        <v>10.02</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="N23" s="4">
-        <v>2.4300000000000002</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="O23" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P23" s="4">
-        <v>2.4300000000000002</v>
+        <v>6.66</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="3" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>148</v>
+        <v>21</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="N24" s="4">
-        <v>0.71</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="O24" s="4">
         <v>1</v>
       </c>
       <c r="P24" s="4">
-        <v>0.71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="N25" s="4">
+        <v>0.71</v>
+      </c>
+      <c r="O25" s="4">
+        <v>1</v>
+      </c>
+      <c r="P25" s="4">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="J25" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K25" s="3" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="M25" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="N25" s="4">
-        <v>4.8499999999999996</v>
-      </c>
-      <c r="O25" s="4">
-        <v>3</v>
-      </c>
-      <c r="P25" s="4">
-        <v>14.55</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>159</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
       <c r="I26" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K26" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="J26" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>160</v>
-      </c>
       <c r="L26" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="M26" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="M26" s="3" t="s">
-        <v>157</v>
-      </c>
       <c r="N26" s="4">
-        <v>3.64</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="O26" s="4">
         <v>3</v>
       </c>
       <c r="P26" s="4">
+        <v>14.55</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="N27" s="4">
+        <v>3.64</v>
+      </c>
+      <c r="O27" s="4">
+        <v>3</v>
+      </c>
+      <c r="P27" s="4">
         <v>10.92</v>
       </c>
     </row>

</xml_diff>